<commit_message>
Artifact Sync with JIRA
Updating legacy artifacts to be synced with JIRA cloud
</commit_message>
<xml_diff>
--- a/Automation Exercise Project/Test Cases/Automation Exercise - Test Case Repository.xlsx
+++ b/Automation Exercise Project/Test Cases/Automation Exercise - Test Case Repository.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="Rdcde8fd1b9134822"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="R0c96b99e96f14988"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R5510328b0c714ad6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="Rb752f6ac4e644024"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="R48bc4ed0262a4b57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R3f1151270f7f4af2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,9 +15,6 @@
     <x:t xml:space="preserve">Automation Exercise | Test Case Repository</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Scope: Authentication, Account Management, Products, Cart, Contact, Navigation &amp; Subscription</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Total Cases</x:t>
   </x:si>
   <x:si>
@@ -102,10 +99,6 @@
     <x:t xml:space="preserve">1. Automation Exercise website is available.
 2. User is not logged in.
 3. Email address has not already been registered.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Name: Kevin Tester
-Email: KevinTheQA@gmail.com</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">1. Open the Automation Exercise website.
@@ -260,11 +253,6 @@
 4. The Signup / Login page is displayed.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Name: Kevin Tester
-Email: KevinTheQA@gmail.com
-Password: ********</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">1. Open the Automation Exercise website.
 2. Click Signup / Login.
 3. Enter valid email address in the Login to your account section.
@@ -333,10 +321,6 @@
     <x:t xml:space="preserve">Verify that login is rejected when a registered email address is entered with an incorrect password</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Email: KevinTheQA@gmail.com
-Password: Incorrect test password</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">1. Open the Automation Exercise website.
 2. Click Signup / Login.
 3. Enter a registered email address in the email field.
@@ -372,10 +356,6 @@
 2. The user has an active registered account.
 3. The user is successfully logged in.
 4. The “Logged in as [username]” indicator is displayed.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Email: KevinTheQA@gmail.com
-Password: *******</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">1. Open the Automation Exercise website.
@@ -1033,7 +1013,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -1114,8 +1094,20 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF0C4A6E"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF92400E"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1167,8 +1159,23 @@
         <x:fgColor rgb="FFF7FBFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE0F2FE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="25">
+  <x:borders count="33">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -1368,12 +1375,124 @@
         <x:color indexed="64"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color indexed="64"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color indexed="64"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color indexed="64"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color indexed="64"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color indexed="64"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color indexed="64"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color indexed="64"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color indexed="64"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color indexed="64"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color indexed="64"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color indexed="64"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color indexed="64"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color indexed="64"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color indexed="64"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color indexed="64"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color indexed="64"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color indexed="64"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color indexed="64"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color indexed="64"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color indexed="64"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFCBD5E1"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="2">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="121">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1542,6 +1661,192 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="11" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="11" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="12" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="12" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="12" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="11" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="11" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="2" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="11" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="12" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="11" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="11" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="13" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="13" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="13" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="13" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -1844,8 +2149,8 @@
       <x:c r="Q1" s="35"/>
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
-      <x:c r="A2" s="36" t="s">
-        <x:v>1</x:v>
+      <x:c r="A2" s="36" t="str">
+        <x:v>Scope: Authentication, Account Management, Products, Cart, Checkout, Contact, Navigation, Reviews &amp; Subscription</x:v>
       </x:c>
       <x:c r="B2" s="36"/>
       <x:c r="C2" s="36"/>
@@ -1866,26 +2171,26 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="46" t="s">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B4" s="47"/>
       <x:c r="C4" s="1"/>
       <x:c r="D4" s="46" t="s">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E4" s="47"/>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="46" t="s">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H4" s="47"/>
       <x:c r="I4" s="1"/>
       <x:c r="J4" s="46" t="s">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K4" s="47"/>
       <x:c r="M4" s="40" t="s">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="N4" s="41"/>
       <x:c r="O4" s="41"/>
@@ -1893,16 +2198,14 @@
     </x:row>
     <x:row r="5" ht="19">
       <x:c r="A5" s="38" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B5" s="39" t="n">
+        <x:f>COUNTA(A8:A107)</x:f>
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B5" s="39"/>
+      <x:c r="C5" s="2"/>
+      <x:c r="D5" s="38" t="n">
+        <x:f>COUNTIF(K8:K107,"Pass")</x:f>
         <x:v>19</x:v>
-      </x:c>
-      <x:c r="C5" s="2" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="D5" s="38" t="n">
-        <x:v>0</x:v>
       </x:c>
       <x:c r="E5" s="39"/>
       <x:c r="F5" s="2"/>
@@ -1914,7 +2217,7 @@
       <x:c r="I5" s="2"/>
       <x:c r="J5" s="38" t="n">
         <x:f>COUNTIF(K8:K107,"Not Run")</x:f>
-        <x:v>0</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="K5" s="39"/>
       <x:c r="M5" s="43"/>
@@ -1924,879 +2227,886 @@
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
       <x:c r="A7" s="14" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" s="15" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B7" s="15" t="s">
+      <x:c r="C7" s="15" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="C7" s="15" t="s">
+      <x:c r="D7" s="15" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="D7" s="15" t="s">
+      <x:c r="E7" s="15" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="E7" s="15" t="s">
+      <x:c r="F7" s="15" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F7" s="15" t="s">
+      <x:c r="G7" s="15" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="G7" s="15" t="s">
+      <x:c r="H7" s="15" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="H7" s="15" t="s">
+      <x:c r="I7" s="15" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="I7" s="15" t="s">
+      <x:c r="J7" s="15" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="J7" s="15" t="s">
+      <x:c r="K7" s="15" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="K7" s="15" t="s">
+      <x:c r="L7" s="15" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="L7" s="15" t="s">
+      <x:c r="M7" s="15" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="M7" s="15" t="s">
+      <x:c r="N7" s="15" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="N7" s="15" t="s">
+      <x:c r="O7" s="15" t="s">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="O7" s="15" t="s">
+      <x:c r="P7" s="15" t="s">
         <x:v>21</x:v>
       </x:c>
-      <x:c r="P7" s="15" t="s">
+      <x:c r="Q7" s="22" t="s">
         <x:v>22</x:v>
-      </x:c>
-      <x:c r="Q7" s="22" t="s">
-        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="232" customHeight="1">
       <x:c r="A8" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="s">
+      <x:c r="C8" s="5" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="s">
+      <x:c r="D8" s="5" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D8" s="5" t="s">
+      <x:c r="E8" s="6" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="E8" s="6" t="s">
+      <x:c r="F8" s="6" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="F8" s="6" t="s">
+      <x:c r="G8" s="6" t="str">
+        <x:v>Name: Kevin Tester
+Email: qa.portfolio@example.com</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="G8" s="6" t="s">
+      <x:c r="I8" s="6" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="H8" s="6" t="s">
+      <x:c r="J8" s="6" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="I8" s="6" t="s">
+      <x:c r="K8" s="5" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="J8" s="6" t="s">
+      <x:c r="L8" s="5" t="s">
         <x:v>33</x:v>
-      </x:c>
-      <x:c r="K8" s="5" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="L8" s="5" t="s">
-        <x:v>35</x:v>
       </x:c>
       <x:c r="M8" s="7">
         <x:v>46223</x:v>
       </x:c>
       <x:c r="N8" s="5" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="O8" s="5" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="P8" s="5" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="O8" s="5" t="s">
+      <x:c r="Q8" s="23" t="s">
         <x:v>37</x:v>
-      </x:c>
-      <x:c r="P8" s="5" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="Q8" s="23" t="s">
-        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="232" customHeight="1">
       <x:c r="A9" s="4" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C9" s="5" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D9" s="5" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="B9" s="5" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="C9" s="5" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="s">
+      <x:c r="F9" s="6" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="E9" s="6" t="s">
+      <x:c r="G9" s="6" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="F9" s="6" t="s">
+      <x:c r="H9" s="6" t="s">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="G9" s="6" t="s">
+      <x:c r="I9" s="6" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="H9" s="6" t="s">
+      <x:c r="J9" s="6" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="I9" s="6" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="J9" s="6" t="s">
-        <x:v>47</x:v>
-      </x:c>
       <x:c r="K9" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L9" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M9" s="7">
         <x:v>46223</x:v>
       </x:c>
       <x:c r="N9" s="5" t="s">
-        <x:v>48</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="O9" s="5" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="P9" s="5" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="Q9" s="23" t="s">
         <x:v>37</x:v>
-      </x:c>
-      <x:c r="P9" s="5" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="Q9" s="23" t="s">
-        <x:v>39</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="232" customHeight="1">
       <x:c r="A10" s="4" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D10" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="C10" s="5" t="s">
+      <x:c r="F10" s="6" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="D10" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E10" s="6" t="s">
+      <x:c r="G10" s="6" t="s">
         <x:v>52</x:v>
       </x:c>
-      <x:c r="F10" s="6" t="s">
+      <x:c r="H10" s="6" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="G10" s="6" t="s">
+      <x:c r="I10" s="6" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="H10" s="6" t="s">
+      <x:c r="J10" s="6" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="I10" s="6" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="J10" s="6" t="s">
-        <x:v>57</x:v>
-      </x:c>
       <x:c r="K10" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L10" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M10" s="7">
         <x:v>46223</x:v>
       </x:c>
       <x:c r="N10" s="5" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="O10" s="5" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="P10" s="5" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="Q10" s="23" t="s">
         <x:v>58</x:v>
-      </x:c>
-      <x:c r="O10" s="5" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="P10" s="5" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="Q10" s="23" t="s">
-        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="232" customHeight="1">
       <x:c r="A11" s="4" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B11" s="5" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C11" s="5" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D11" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="B11" s="5" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="C11" s="5" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="D11" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E11" s="6" t="s">
+      <x:c r="H11" s="6" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="F11" s="6" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="G11" s="6" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="H11" s="6" t="s">
-        <x:v>64</x:v>
-      </x:c>
       <x:c r="I11" s="6" t="s">
-        <x:v>56</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="J11" s="6" t="s">
-        <x:v>57</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="K11" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L11" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M11" s="7">
         <x:v>46223</x:v>
       </x:c>
       <x:c r="N11" s="5" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="O11" s="5" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="P11" s="5" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="Q11" s="23" t="s">
         <x:v>65</x:v>
-      </x:c>
-      <x:c r="O11" s="5" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="P11" s="5" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="Q11" s="23" t="s">
-        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="232" customHeight="1">
       <x:c r="A12" s="4" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B12" s="5" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="C12" s="5" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D12" s="5" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="s">
+      <x:c r="F12" s="6" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C12" s="5" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="E12" s="6" t="s">
+      <x:c r="G12" s="6" t="str">
+        <x:v>Name: Kevin Tester
+Email: qa.portfolio@example.com
+Password: ********</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="F12" s="6" t="s">
+      <x:c r="I12" s="6" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="G12" s="6" t="s">
+      <x:c r="J12" s="6" t="s">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="H12" s="6" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="I12" s="6" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="J12" s="6" t="s">
-        <x:v>75</x:v>
-      </x:c>
       <x:c r="K12" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L12" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M12" s="7">
         <x:v>46224</x:v>
       </x:c>
       <x:c r="N12" s="5" t="s">
-        <x:v>76</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="O12" s="5" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P12" s="5" t="s">
-        <x:v>77</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="Q12" s="23" t="s">
-        <x:v>78</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="232" customHeight="1">
       <x:c r="A13" s="4" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="B13" s="5" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="C13" s="5" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="D13" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="s">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="B13" s="5" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="C13" s="5" t="s">
+      <x:c r="G13" s="6" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="D13" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E13" s="6" t="s">
+      <x:c r="H13" s="6" t="s">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="F13" s="6" t="s">
+      <x:c r="I13" s="6" t="s">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="G13" s="6" t="s">
+      <x:c r="J13" s="6" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="H13" s="6" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="I13" s="6" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="J13" s="6" t="s">
-        <x:v>86</x:v>
-      </x:c>
       <x:c r="K13" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L13" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M13" s="7">
         <x:v>46224</x:v>
       </x:c>
       <x:c r="N13" s="5" t="s">
-        <x:v>87</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="O13" s="5" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P13" s="5" t="s">
-        <x:v>88</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="Q13" s="23" t="s">
-        <x:v>89</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="232" customHeight="1">
       <x:c r="A14" s="4" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="B14" s="5" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="C14" s="5" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D14" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E14" s="6" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="F14" s="6" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="G14" s="6" t="str">
+        <x:v>Email: qa.portfolio@example.com
+Password: Incorrect test password</x:v>
+      </x:c>
+      <x:c r="H14" s="6" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="I14" s="6" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="B14" s="5" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="D14" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E14" s="6" t="s">
+      <x:c r="J14" s="6" t="s">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="F14" s="6" t="s">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="G14" s="6" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="H14" s="6" t="s">
-        <x:v>93</x:v>
-      </x:c>
-      <x:c r="I14" s="6" t="s">
-        <x:v>94</x:v>
-      </x:c>
-      <x:c r="J14" s="6" t="s">
-        <x:v>95</x:v>
-      </x:c>
       <x:c r="K14" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L14" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M14" s="7">
         <x:v>46224</x:v>
       </x:c>
       <x:c r="N14" s="5" t="s">
-        <x:v>96</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="O14" s="5" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P14" s="5" t="s">
-        <x:v>97</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="Q14" s="23" t="s">
-        <x:v>98</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="232" customHeight="1">
       <x:c r="A15" s="4" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B15" s="5" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="C15" s="5" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D15" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E15" s="6" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="F15" s="6" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="G15" s="6" t="str">
+        <x:v>Email: qa.portfolio@example.com
+Password: *******</x:v>
+      </x:c>
+      <x:c r="H15" s="6" t="s">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="B15" s="5" t="s">
+      <x:c r="I15" s="6" t="s">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="C15" s="5" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D15" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E15" s="6" t="s">
+      <x:c r="J15" s="6" t="s">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="F15" s="6" t="s">
+      <x:c r="K15" s="5" t="s">
         <x:v>102</x:v>
       </x:c>
-      <x:c r="G15" s="6" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="H15" s="6" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="I15" s="6" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="J15" s="6" t="s">
-        <x:v>106</x:v>
-      </x:c>
-      <x:c r="K15" s="5" t="s">
-        <x:v>107</x:v>
-      </x:c>
       <x:c r="L15" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M15" s="7">
         <x:v>46232</x:v>
       </x:c>
       <x:c r="N15" s="5" t="s">
-        <x:v>108</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="O15" s="28" t="s">
-        <x:v>109</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="P15" s="5" t="s">
-        <x:v>110</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="Q15" s="23" t="s">
-        <x:v>111</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="232" customHeight="1">
       <x:c r="A16" s="4" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="B16" s="5" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="C16" s="5" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D16" s="5" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E16" s="6" t="s">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="str">
+        <x:v>Email: qa.portfolio@example.com
+Password: *******</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="s">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="I16" s="6" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="s">
+      <x:c r="J16" s="6" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="C16" s="5" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D16" s="5" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="E16" s="6" t="s">
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="F16" s="6" t="s">
-        <x:v>115</x:v>
-      </x:c>
-      <x:c r="G16" s="6" t="s">
-        <x:v>103</x:v>
-      </x:c>
-      <x:c r="H16" s="6" t="s">
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="I16" s="6" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="J16" s="6" t="s">
-        <x:v>118</x:v>
-      </x:c>
       <x:c r="K16" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L16" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M16" s="7">
         <x:v>46232</x:v>
       </x:c>
       <x:c r="N16" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="O16" s="5" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P16" s="5" t="s">
-        <x:v>120</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="Q16" s="23" t="s">
-        <x:v>121</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="232" customHeight="1">
       <x:c r="A17" s="4" t="s">
-        <x:v>122</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B17" s="5" t="s">
-        <x:v>113</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C17" s="5" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D17" s="5" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D17" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
       <x:c r="E17" s="6" t="s">
-        <x:v>123</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="F17" s="6" t="s">
-        <x:v>124</x:v>
-      </x:c>
-      <x:c r="G17" s="6" t="s">
-        <x:v>103</x:v>
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="G17" s="6" t="str">
+        <x:v>Email: qa.portfolio@example.com
+Password: *******</x:v>
       </x:c>
       <x:c r="H17" s="6" t="s">
-        <x:v>125</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="I17" s="6" t="s">
-        <x:v>126</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="J17" s="6" t="s">
-        <x:v>126</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="K17" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L17" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M17" s="7">
         <x:v>46232</x:v>
       </x:c>
       <x:c r="N17" s="5" t="s">
-        <x:v>127</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="O17" s="5" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P17" s="5" t="s">
-        <x:v>128</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="Q17" s="23" t="s">
-        <x:v>129</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="142" customHeight="1">
       <x:c r="A18" s="4" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C18" s="5" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D18" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E18" s="6" t="s">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="F18" s="6" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="G18" s="6" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="H18" s="6" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="I18" s="6" t="s">
         <x:v>130</x:v>
       </x:c>
-      <x:c r="B18" s="5" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="C18" s="5" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="D18" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E18" s="6" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="F18" s="6" t="s">
-        <x:v>132</x:v>
-      </x:c>
-      <x:c r="G18" s="6" t="s">
-        <x:v>133</x:v>
-      </x:c>
-      <x:c r="H18" s="6" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="I18" s="6" t="s">
-        <x:v>135</x:v>
-      </x:c>
       <x:c r="J18" s="6" t="s">
-        <x:v>135</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="K18" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L18" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M18" s="7">
         <x:v>46233</x:v>
       </x:c>
       <x:c r="N18" s="28" t="s">
-        <x:v>136</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="O18" s="5" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P18" s="5" t="s">
-        <x:v>137</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="Q18" s="23" t="s">
-        <x:v>138</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="142" customHeight="1">
       <x:c r="A19" s="4" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="B19" s="5" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="C19" s="5" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D19" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E19" s="6" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="F19" s="6" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="G19" s="6" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="H19" s="6" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="I19" s="6" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="B19" s="5" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="C19" s="5" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="D19" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E19" s="6" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="F19" s="6" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="G19" s="6" t="s">
-        <x:v>142</x:v>
-      </x:c>
-      <x:c r="H19" s="6" t="s">
-        <x:v>143</x:v>
-      </x:c>
-      <x:c r="I19" s="6" t="s">
-        <x:v>144</x:v>
-      </x:c>
       <x:c r="J19" s="6" t="s">
-        <x:v>144</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="K19" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L19" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M19" s="7">
         <x:v>46233</x:v>
       </x:c>
       <x:c r="N19" s="28" t="s">
-        <x:v>145</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="O19" s="5" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P19" s="5" t="s">
-        <x:v>146</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="Q19" s="23" t="s">
-        <x:v>98</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="142" customHeight="1">
       <x:c r="A20" s="4" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="B20" s="5" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="C20" s="5" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D20" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E20" s="6" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="F20" s="6" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="G20" s="6" t="s">
+        <x:v>146</x:v>
+      </x:c>
+      <x:c r="H20" s="6" t="s">
         <x:v>147</x:v>
       </x:c>
-      <x:c r="B20" s="5" t="s">
+      <x:c r="I20" s="6" t="s">
         <x:v>148</x:v>
       </x:c>
-      <x:c r="C20" s="5" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D20" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E20" s="6" t="s">
-        <x:v>149</x:v>
-      </x:c>
-      <x:c r="F20" s="6" t="s">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="G20" s="6" t="s">
-        <x:v>151</x:v>
-      </x:c>
-      <x:c r="H20" s="6" t="s">
-        <x:v>152</x:v>
-      </x:c>
-      <x:c r="I20" s="6" t="s">
-        <x:v>153</x:v>
-      </x:c>
       <x:c r="J20" s="6" t="s">
-        <x:v>153</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="K20" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L20" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M20" s="7">
         <x:v>46233</x:v>
       </x:c>
       <x:c r="N20" s="28" t="s">
-        <x:v>154</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="O20" s="5" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P20" s="5" t="s">
-        <x:v>155</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="Q20" s="23" t="s">
-        <x:v>156</x:v>
+        <x:v>151</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="142" customHeight="1">
       <x:c r="A21" s="4" t="s">
+        <x:v>152</x:v>
+      </x:c>
+      <x:c r="B21" s="5" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="C21" s="5" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D21" s="5" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E21" s="6" t="s">
+        <x:v>153</x:v>
+      </x:c>
+      <x:c r="F21" s="6" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="G21" s="6" t="s">
+        <x:v>155</x:v>
+      </x:c>
+      <x:c r="H21" s="6" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="I21" s="6" t="s">
         <x:v>157</x:v>
       </x:c>
-      <x:c r="B21" s="5" t="s">
-        <x:v>148</x:v>
-      </x:c>
-      <x:c r="C21" s="5" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D21" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="E21" s="6" t="s">
-        <x:v>158</x:v>
-      </x:c>
-      <x:c r="F21" s="6" t="s">
-        <x:v>159</x:v>
-      </x:c>
-      <x:c r="G21" s="6" t="s">
-        <x:v>160</x:v>
-      </x:c>
-      <x:c r="H21" s="6" t="s">
-        <x:v>161</x:v>
-      </x:c>
-      <x:c r="I21" s="6" t="s">
-        <x:v>162</x:v>
-      </x:c>
       <x:c r="J21" s="6" t="s">
-        <x:v>162</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="K21" s="5" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L21" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M21" s="7">
         <x:v>46233</x:v>
       </x:c>
       <x:c r="N21" s="28" t="s">
-        <x:v>163</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="O21" s="5" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P21" s="5" t="s">
-        <x:v>164</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="Q21" s="23" t="s">
-        <x:v>165</x:v>
+        <x:v>160</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="142" customHeight="1">
       <x:c r="A22" s="4" t="s">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="B22" s="5" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="C22" s="5" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D22" s="5" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="E22" s="6" t="s">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="F22" s="6" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="G22" s="6" t="s">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="H22" s="6" t="s">
         <x:v>166</x:v>
       </x:c>
-      <x:c r="B22" s="5" t="s">
+      <x:c r="I22" s="6" t="s">
         <x:v>167</x:v>
       </x:c>
-      <x:c r="C22" s="5" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D22" s="5" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="E22" s="6" t="s">
+      <x:c r="J22" s="6" t="s">
         <x:v>168</x:v>
       </x:c>
-      <x:c r="F22" s="6" t="s">
-        <x:v>169</x:v>
-      </x:c>
-      <x:c r="G22" s="6" t="s">
-        <x:v>170</x:v>
-      </x:c>
-      <x:c r="H22" s="6" t="s">
-        <x:v>171</x:v>
-      </x:c>
-      <x:c r="I22" s="6" t="s">
-        <x:v>172</x:v>
-      </x:c>
-      <x:c r="J22" s="6" t="s">
-        <x:v>173</x:v>
-      </x:c>
       <x:c r="K22" s="5" t="s">
-        <x:v>107</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="L22" s="5" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M22" s="7">
         <x:v>46233</x:v>
       </x:c>
       <x:c r="N22" s="28" t="s">
-        <x:v>174</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="O22" s="5" t="str">
         <x:v>AE-BUG-003</x:v>
       </x:c>
       <x:c r="P22" s="5" t="s">
-        <x:v>175</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="Q22" s="23" t="s">
-        <x:v>176</x:v>
+        <x:v>171</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="142" customHeight="1">
       <x:c r="A23" s="4" t="s">
-        <x:v>177</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="B23" s="5" t="s">
-        <x:v>167</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="C23" s="5" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D23" s="5" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D23" s="5" t="s">
-        <x:v>27</x:v>
-      </x:c>
       <x:c r="E23" s="6" t="s">
-        <x:v>178</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="F23" s="6" t="s">
-        <x:v>150</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="G23" s="6" t="s">
-        <x:v>179</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="H23" s="6" t="s">
-        <x:v>180</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="I23" s="6" t="s">
-        <x:v>181</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="J23" s="6" t="str">
         <x:v>The selected product was displayed in the cart with quantity 4, and the line total equaled the unit price multiplied by 4.</x:v>
@@ -2825,515 +3135,913 @@
     </x:row>
     <x:row r="24" ht="142" customHeight="1">
       <x:c r="A24" s="8" t="s">
-        <x:v>182</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B24" s="9" t="s">
-        <x:v>167</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="C24" s="9" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D24" s="9" t="s">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D24" s="9" t="s">
-        <x:v>27</x:v>
-      </x:c>
       <x:c r="E24" s="10" t="s">
-        <x:v>183</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="F24" s="10" t="s">
-        <x:v>150</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="G24" s="10" t="s">
-        <x:v>184</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="H24" s="10" t="s">
-        <x:v>185</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="I24" s="10" t="s">
-        <x:v>186</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="J24" s="10" t="s">
-        <x:v>186</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="K24" s="9" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L24" s="9" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M24" s="11">
         <x:v>46234</x:v>
       </x:c>
       <x:c r="N24" s="29" t="s">
-        <x:v>187</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="O24" s="9" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P24" s="9" t="s">
-        <x:v>188</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="Q24" s="24" t="s">
-        <x:v>189</x:v>
+        <x:v>184</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="260" customHeight="1">
       <x:c r="A25" s="33" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="B25" s="33" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="C25" s="33" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D25" s="33" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="E25" s="32" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="F25" s="32" t="s">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="G25" s="32" t="s">
         <x:v>190</x:v>
       </x:c>
-      <x:c r="B25" s="33" t="s">
+      <x:c r="H25" s="32" t="s">
         <x:v>191</x:v>
       </x:c>
-      <x:c r="C25" s="33" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D25" s="33" t="s">
+      <x:c r="I25" s="32" t="s">
         <x:v>192</x:v>
       </x:c>
-      <x:c r="E25" s="32" t="s">
-        <x:v>193</x:v>
-      </x:c>
-      <x:c r="F25" s="32" t="s">
-        <x:v>194</x:v>
-      </x:c>
-      <x:c r="G25" s="32" t="s">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="H25" s="32" t="s">
-        <x:v>196</x:v>
-      </x:c>
-      <x:c r="I25" s="32" t="s">
-        <x:v>197</x:v>
-      </x:c>
       <x:c r="J25" s="32" t="s">
-        <x:v>197</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="K25" s="33" t="str">
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="L25" s="33" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M25" s="34">
         <x:v>46235</x:v>
       </x:c>
       <x:c r="N25" s="28" t="s">
-        <x:v>198</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="O25" s="33" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P25" s="32" t="s">
-        <x:v>199</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="Q25" s="33" t="s">
-        <x:v>200</x:v>
+        <x:v>195</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="150" customHeight="1">
       <x:c r="A26" s="33" t="s">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="B26" s="33" t="s">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="C26" s="33" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D26" s="33" t="s">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="E26" s="32" t="s">
+        <x:v>199</x:v>
+      </x:c>
+      <x:c r="F26" s="32" t="s">
+        <x:v>200</x:v>
+      </x:c>
+      <x:c r="G26" s="32" t="s">
         <x:v>201</x:v>
       </x:c>
-      <x:c r="B26" s="33" t="s">
+      <x:c r="H26" s="32" t="s">
         <x:v>202</x:v>
       </x:c>
-      <x:c r="C26" s="33" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D26" s="33" t="s">
+      <x:c r="I26" s="32" t="s">
         <x:v>203</x:v>
       </x:c>
-      <x:c r="E26" s="32" t="s">
-        <x:v>204</x:v>
-      </x:c>
-      <x:c r="F26" s="32" t="s">
-        <x:v>205</x:v>
-      </x:c>
-      <x:c r="G26" s="32" t="s">
-        <x:v>206</x:v>
-      </x:c>
-      <x:c r="H26" s="32" t="s">
-        <x:v>207</x:v>
-      </x:c>
-      <x:c r="I26" s="32" t="s">
-        <x:v>208</x:v>
-      </x:c>
       <x:c r="J26" s="32" t="s">
-        <x:v>208</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="K26" s="33" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L26" s="33" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M26" s="34">
         <x:v>46235</x:v>
       </x:c>
       <x:c r="N26" s="28" t="s">
-        <x:v>209</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="O26" s="33" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P26" s="32" t="s">
-        <x:v>210</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="Q26" s="33" t="s">
-        <x:v>211</x:v>
+        <x:v>206</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="190" customHeight="1">
       <x:c r="A27" s="33" t="s">
+        <x:v>207</x:v>
+      </x:c>
+      <x:c r="B27" s="33" t="s">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="C27" s="33" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D27" s="33" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="E27" s="32" t="s">
+        <x:v>209</x:v>
+      </x:c>
+      <x:c r="F27" s="32" t="s">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="G27" s="32" t="s">
+        <x:v>211</x:v>
+      </x:c>
+      <x:c r="H27" s="32" t="s">
         <x:v>212</x:v>
       </x:c>
-      <x:c r="B27" s="33" t="s">
+      <x:c r="I27" s="32" t="s">
         <x:v>213</x:v>
       </x:c>
-      <x:c r="C27" s="33" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="D27" s="33" t="s">
-        <x:v>192</x:v>
-      </x:c>
-      <x:c r="E27" s="32" t="s">
-        <x:v>214</x:v>
-      </x:c>
-      <x:c r="F27" s="32" t="s">
-        <x:v>215</x:v>
-      </x:c>
-      <x:c r="G27" s="32" t="s">
-        <x:v>216</x:v>
-      </x:c>
-      <x:c r="H27" s="32" t="s">
-        <x:v>217</x:v>
-      </x:c>
-      <x:c r="I27" s="32" t="s">
-        <x:v>218</x:v>
-      </x:c>
       <x:c r="J27" s="32" t="s">
-        <x:v>218</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="K27" s="33" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L27" s="33" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M27" s="34">
         <x:v>46235</x:v>
       </x:c>
       <x:c r="N27" s="28" t="s">
-        <x:v>219</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="O27" s="33" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P27" s="32" t="s">
-        <x:v>210</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="Q27" s="33" t="s">
-        <x:v>220</x:v>
+        <x:v>215</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="210" customHeight="1">
       <x:c r="A28" s="33" t="s">
-        <x:v>221</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="B28" s="33" t="s">
-        <x:v>213</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="C28" s="33" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D28" s="33" t="s">
-        <x:v>192</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="E28" s="32" t="s">
-        <x:v>222</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="F28" s="32" t="s">
-        <x:v>215</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="G28" s="32" t="s">
-        <x:v>223</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="H28" s="32" t="s">
-        <x:v>224</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="I28" s="32" t="s">
-        <x:v>225</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="J28" s="32" t="s">
-        <x:v>225</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="K28" s="33" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="L28" s="33" t="s">
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="M28" s="34">
         <x:v>46235</x:v>
       </x:c>
       <x:c r="N28" s="28" t="s">
-        <x:v>226</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="O28" s="33" t="s">
-        <x:v>37</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="P28" s="32" t="s">
-        <x:v>210</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="Q28" s="33" t="s">
-        <x:v>227</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="30"/>
-      <x:c r="B29" s="30"/>
-      <x:c r="C29" s="30"/>
-      <x:c r="D29" s="30"/>
-      <x:c r="E29" s="30"/>
-      <x:c r="F29" s="30"/>
-      <x:c r="G29" s="30"/>
-      <x:c r="H29" s="30"/>
-      <x:c r="I29" s="30"/>
-      <x:c r="J29" s="30"/>
-      <x:c r="K29" s="30"/>
-      <x:c r="L29" s="30"/>
-      <x:c r="M29" s="31"/>
-      <x:c r="N29" s="30"/>
-      <x:c r="O29" s="30"/>
-      <x:c r="P29" s="30"/>
-      <x:c r="Q29" s="30"/>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="30"/>
-      <x:c r="B30" s="30"/>
-      <x:c r="C30" s="30"/>
-      <x:c r="D30" s="30"/>
-      <x:c r="E30" s="30"/>
-      <x:c r="F30" s="30"/>
-      <x:c r="G30" s="30"/>
-      <x:c r="H30" s="30"/>
-      <x:c r="I30" s="30"/>
-      <x:c r="J30" s="30"/>
-      <x:c r="K30" s="30"/>
-      <x:c r="L30" s="30"/>
-      <x:c r="M30" s="31"/>
-      <x:c r="N30" s="30"/>
-      <x:c r="O30" s="30"/>
-      <x:c r="P30" s="30"/>
-      <x:c r="Q30" s="30"/>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="30"/>
-      <x:c r="B31" s="30"/>
-      <x:c r="C31" s="30"/>
-      <x:c r="D31" s="30"/>
-      <x:c r="E31" s="30"/>
-      <x:c r="F31" s="30"/>
-      <x:c r="G31" s="30"/>
-      <x:c r="H31" s="30"/>
-      <x:c r="I31" s="30"/>
-      <x:c r="J31" s="30"/>
-      <x:c r="K31" s="30"/>
-      <x:c r="L31" s="30"/>
-      <x:c r="M31" s="31"/>
-      <x:c r="N31" s="30"/>
-      <x:c r="O31" s="30"/>
-      <x:c r="P31" s="30"/>
-      <x:c r="Q31" s="30"/>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="30"/>
-      <x:c r="B32" s="30"/>
-      <x:c r="C32" s="30"/>
-      <x:c r="D32" s="30"/>
-      <x:c r="E32" s="30"/>
-      <x:c r="F32" s="30"/>
-      <x:c r="G32" s="30"/>
-      <x:c r="H32" s="30"/>
-      <x:c r="I32" s="30"/>
-      <x:c r="J32" s="30"/>
-      <x:c r="K32" s="30"/>
-      <x:c r="L32" s="30"/>
-      <x:c r="M32" s="31"/>
-      <x:c r="N32" s="30"/>
-      <x:c r="O32" s="30"/>
-      <x:c r="P32" s="30"/>
-      <x:c r="Q32" s="30"/>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="30"/>
-      <x:c r="B33" s="30"/>
-      <x:c r="C33" s="30"/>
-      <x:c r="D33" s="30"/>
-      <x:c r="E33" s="30"/>
-      <x:c r="F33" s="30"/>
-      <x:c r="G33" s="30"/>
-      <x:c r="H33" s="30"/>
-      <x:c r="I33" s="30"/>
-      <x:c r="J33" s="30"/>
-      <x:c r="K33" s="30"/>
-      <x:c r="L33" s="30"/>
-      <x:c r="M33" s="31"/>
-      <x:c r="N33" s="30"/>
-      <x:c r="O33" s="30"/>
-      <x:c r="P33" s="30"/>
-      <x:c r="Q33" s="30"/>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="30"/>
-      <x:c r="B34" s="30"/>
-      <x:c r="C34" s="30"/>
-      <x:c r="D34" s="30"/>
-      <x:c r="E34" s="30"/>
-      <x:c r="F34" s="30"/>
-      <x:c r="G34" s="30"/>
-      <x:c r="H34" s="30"/>
-      <x:c r="I34" s="30"/>
-      <x:c r="J34" s="30"/>
-      <x:c r="K34" s="30"/>
-      <x:c r="L34" s="30"/>
-      <x:c r="M34" s="31"/>
-      <x:c r="N34" s="30"/>
-      <x:c r="O34" s="30"/>
-      <x:c r="P34" s="30"/>
-      <x:c r="Q34" s="30"/>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="30"/>
-      <x:c r="B35" s="30"/>
-      <x:c r="C35" s="30"/>
-      <x:c r="D35" s="30"/>
-      <x:c r="E35" s="30"/>
-      <x:c r="F35" s="30"/>
-      <x:c r="G35" s="30"/>
-      <x:c r="H35" s="30"/>
-      <x:c r="I35" s="30"/>
-      <x:c r="J35" s="30"/>
-      <x:c r="K35" s="30"/>
-      <x:c r="L35" s="30"/>
-      <x:c r="M35" s="31"/>
-      <x:c r="N35" s="30"/>
-      <x:c r="O35" s="30"/>
-      <x:c r="P35" s="30"/>
-      <x:c r="Q35" s="30"/>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="30"/>
-      <x:c r="B36" s="30"/>
-      <x:c r="C36" s="30"/>
-      <x:c r="D36" s="30"/>
-      <x:c r="E36" s="30"/>
-      <x:c r="F36" s="30"/>
-      <x:c r="G36" s="30"/>
-      <x:c r="H36" s="30"/>
-      <x:c r="I36" s="30"/>
-      <x:c r="J36" s="30"/>
-      <x:c r="K36" s="30"/>
-      <x:c r="L36" s="30"/>
-      <x:c r="M36" s="31"/>
-      <x:c r="N36" s="30"/>
-      <x:c r="O36" s="30"/>
-      <x:c r="P36" s="30"/>
-      <x:c r="Q36" s="30"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="30"/>
-      <x:c r="B37" s="30"/>
-      <x:c r="C37" s="30"/>
-      <x:c r="D37" s="30"/>
-      <x:c r="E37" s="30"/>
-      <x:c r="F37" s="30"/>
-      <x:c r="G37" s="30"/>
-      <x:c r="H37" s="30"/>
-      <x:c r="I37" s="30"/>
-      <x:c r="J37" s="30"/>
-      <x:c r="K37" s="30"/>
-      <x:c r="L37" s="30"/>
-      <x:c r="M37" s="31"/>
-      <x:c r="N37" s="30"/>
-      <x:c r="O37" s="30"/>
-      <x:c r="P37" s="30"/>
-      <x:c r="Q37" s="30"/>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="30"/>
-      <x:c r="B38" s="30"/>
-      <x:c r="C38" s="30"/>
-      <x:c r="D38" s="30"/>
-      <x:c r="E38" s="30"/>
-      <x:c r="F38" s="30"/>
-      <x:c r="G38" s="30"/>
-      <x:c r="H38" s="30"/>
-      <x:c r="I38" s="30"/>
-      <x:c r="J38" s="30"/>
-      <x:c r="K38" s="30"/>
-      <x:c r="L38" s="30"/>
-      <x:c r="M38" s="31"/>
-      <x:c r="N38" s="30"/>
-      <x:c r="O38" s="30"/>
-      <x:c r="P38" s="30"/>
-      <x:c r="Q38" s="30"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="30"/>
-      <x:c r="B39" s="30"/>
-      <x:c r="C39" s="30"/>
-      <x:c r="D39" s="30"/>
-      <x:c r="E39" s="30"/>
-      <x:c r="F39" s="30"/>
-      <x:c r="G39" s="30"/>
-      <x:c r="H39" s="30"/>
-      <x:c r="I39" s="30"/>
-      <x:c r="J39" s="30"/>
-      <x:c r="K39" s="30"/>
-      <x:c r="L39" s="30"/>
-      <x:c r="M39" s="31"/>
-      <x:c r="N39" s="30"/>
-      <x:c r="O39" s="30"/>
-      <x:c r="P39" s="30"/>
-      <x:c r="Q39" s="30"/>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="30"/>
-      <x:c r="B40" s="30"/>
-      <x:c r="C40" s="30"/>
-      <x:c r="D40" s="30"/>
-      <x:c r="E40" s="30"/>
-      <x:c r="F40" s="30"/>
-      <x:c r="G40" s="30"/>
-      <x:c r="H40" s="30"/>
-      <x:c r="I40" s="30"/>
-      <x:c r="J40" s="30"/>
-      <x:c r="K40" s="30"/>
-      <x:c r="L40" s="30"/>
-      <x:c r="M40" s="31"/>
-      <x:c r="N40" s="30"/>
-      <x:c r="O40" s="30"/>
-      <x:c r="P40" s="30"/>
-      <x:c r="Q40" s="30"/>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="30"/>
-      <x:c r="B41" s="30"/>
-      <x:c r="C41" s="30"/>
-      <x:c r="D41" s="30"/>
-      <x:c r="E41" s="30"/>
-      <x:c r="F41" s="30"/>
-      <x:c r="G41" s="30"/>
-      <x:c r="H41" s="30"/>
-      <x:c r="I41" s="30"/>
-      <x:c r="J41" s="30"/>
-      <x:c r="K41" s="30"/>
-      <x:c r="L41" s="30"/>
-      <x:c r="M41" s="31"/>
-      <x:c r="N41" s="30"/>
-      <x:c r="O41" s="30"/>
-      <x:c r="P41" s="30"/>
-      <x:c r="Q41" s="30"/>
+        <x:v>222</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="112.5" customHeight="1">
+      <x:c r="A29" s="111" t="str">
+        <x:v>AE-SIGNUP-006</x:v>
+      </x:c>
+      <x:c r="B29" s="88" t="str">
+        <x:v>Signup</x:v>
+      </x:c>
+      <x:c r="C29" s="88" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D29" s="88" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="E29" s="84" t="str">
+        <x:v>Verify the complete registration workflow including optional subscription selections</x:v>
+      </x:c>
+      <x:c r="F29" s="84" t="str">
+        <x:v>Automation Exercise is available; user is logged out; a unique disposable email is available.</x:v>
+      </x:c>
+      <x:c r="G29" s="84" t="str">
+        <x:v>Unique QA name and email; safe account details; newsletter and special-offer selections enabled.</x:v>
+      </x:c>
+      <x:c r="H29" s="84" t="str">
+        <x:v>1. Open automationexercise.com and select Signup / Login.
+2. Start signup with a valid name and unique email.
+3. Complete all required account fields.
+4. Select Sign up for our newsletter and Receive special offers from our partners.
+5. Create the account and continue to the home page.
+6. Verify Logged in as is displayed.
+7. Delete the disposable account as cleanup.</x:v>
+      </x:c>
+      <x:c r="I29" s="84" t="str">
+        <x:v>The account is created successfully, the user is authenticated, optional selections do not block registration, and cleanup succeeds.</x:v>
+      </x:c>
+      <x:c r="J29" s="84" t="str"/>
+      <x:c r="K29" s="118" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L29" s="88" t="str"/>
+      <x:c r="M29" s="89" t="str"/>
+      <x:c r="N29" s="88" t="str"/>
+      <x:c r="O29" s="88" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P29" s="84" t="str">
+        <x:v>Jira AEQA-106; linked to AEQA-1. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q29" s="86" t="str">
+        <x:v>REQ-AUTH-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="112.5" customHeight="1">
+      <x:c r="A30" s="112" t="str">
+        <x:v>AE-ORDER-001</x:v>
+      </x:c>
+      <x:c r="B30" s="95" t="str">
+        <x:v>Checkout</x:v>
+      </x:c>
+      <x:c r="C30" s="95" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D30" s="95" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="E30" s="91" t="str">
+        <x:v>Verify an order can be placed after registering during checkout</x:v>
+      </x:c>
+      <x:c r="F30" s="91" t="str">
+        <x:v>Automation Exercise is available; user is logged out; cart is empty; a unique email is available.</x:v>
+      </x:c>
+      <x:c r="G30" s="91" t="str">
+        <x:v>One in-stock product; unique QA account data; safe test payment data supplied by the site scenario.</x:v>
+      </x:c>
+      <x:c r="H30" s="91" t="str">
+        <x:v>1. Add a product to the cart.
+2. Open Cart and select Proceed To Checkout.
+3. Choose Register / Login.
+4. Create and confirm a new account.
+5. Return to Cart and proceed to checkout.
+6. Verify address and order details.
+7. Enter an order comment and place the order.
+8. Enter test payment details and confirm.
+9. Verify the success message and delete the disposable account.</x:v>
+      </x:c>
+      <x:c r="I30" s="91" t="str">
+        <x:v>The newly registered user completes checkout and sees the order success confirmation.</x:v>
+      </x:c>
+      <x:c r="J30" s="91" t="str"/>
+      <x:c r="K30" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L30" s="95" t="str"/>
+      <x:c r="M30" s="96" t="str"/>
+      <x:c r="N30" s="95" t="str"/>
+      <x:c r="O30" s="95" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P30" s="91" t="str">
+        <x:v>Jira AEQA-107; linked to AEQA-14. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q30" s="93" t="str">
+        <x:v>REQ-ORDER-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="112.5" customHeight="1">
+      <x:c r="A31" s="113" t="str">
+        <x:v>AE-ORDER-002</x:v>
+      </x:c>
+      <x:c r="B31" s="102" t="str">
+        <x:v>Checkout</x:v>
+      </x:c>
+      <x:c r="C31" s="102" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D31" s="102" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="E31" s="98" t="str">
+        <x:v>Verify an order can be placed after registering before checkout</x:v>
+      </x:c>
+      <x:c r="F31" s="98" t="str">
+        <x:v>Automation Exercise is available; user is logged out; a unique email is available.</x:v>
+      </x:c>
+      <x:c r="G31" s="98" t="str">
+        <x:v>Unique QA account; one in-stock product; safe test payment data.</x:v>
+      </x:c>
+      <x:c r="H31" s="98" t="str">
+        <x:v>1. Register a new account from Signup / Login.
+2. Confirm Logged in as is displayed.
+3. Add a product to the cart.
+4. Proceed to checkout.
+5. Verify address and order details.
+6. Place the order and provide test payment details.
+7. Confirm the order and verify success.
+8. Delete the disposable account.</x:v>
+      </x:c>
+      <x:c r="I31" s="98" t="str">
+        <x:v>A user registered before shopping can place the order successfully and receives confirmation.</x:v>
+      </x:c>
+      <x:c r="J31" s="98" t="str"/>
+      <x:c r="K31" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L31" s="102" t="str"/>
+      <x:c r="M31" s="103" t="str"/>
+      <x:c r="N31" s="102" t="str"/>
+      <x:c r="O31" s="102" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P31" s="98" t="str">
+        <x:v>Jira AEQA-108; linked to AEQA-15. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q31" s="100" t="str">
+        <x:v>REQ-ORDER-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="112.5" customHeight="1">
+      <x:c r="A32" s="112" t="str">
+        <x:v>AE-ORDER-003</x:v>
+      </x:c>
+      <x:c r="B32" s="95" t="str">
+        <x:v>Checkout</x:v>
+      </x:c>
+      <x:c r="C32" s="95" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D32" s="95" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="E32" s="91" t="str">
+        <x:v>Verify an existing user can log in before checkout and place an order</x:v>
+      </x:c>
+      <x:c r="F32" s="91" t="str">
+        <x:v>A dedicated Automation Exercise QA account exists and is logged out.</x:v>
+      </x:c>
+      <x:c r="G32" s="91" t="str">
+        <x:v>Valid QA credentials; one in-stock product; safe test payment data.</x:v>
+      </x:c>
+      <x:c r="H32" s="91" t="str">
+        <x:v>1. Open Signup / Login and authenticate with the QA account.
+2. Verify Logged in as is displayed.
+3. Add a product to the cart and proceed to checkout.
+4. Verify address and order details.
+5. Place the order and provide test payment details.
+6. Confirm the order.</x:v>
+      </x:c>
+      <x:c r="I32" s="91" t="str">
+        <x:v>The authenticated user completes checkout and sees the order success confirmation.</x:v>
+      </x:c>
+      <x:c r="J32" s="91" t="str"/>
+      <x:c r="K32" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L32" s="95" t="str"/>
+      <x:c r="M32" s="96" t="str"/>
+      <x:c r="N32" s="95" t="str"/>
+      <x:c r="O32" s="95" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P32" s="91" t="str">
+        <x:v>Jira AEQA-109; linked to AEQA-16. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q32" s="93" t="str">
+        <x:v>REQ-ORDER-003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="112.5" customHeight="1">
+      <x:c r="A33" s="113" t="str">
+        <x:v>AE-CATALOG-001</x:v>
+      </x:c>
+      <x:c r="B33" s="102" t="str">
+        <x:v>Products</x:v>
+      </x:c>
+      <x:c r="C33" s="102" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D33" s="102" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E33" s="98" t="str">
+        <x:v>Verify category and subcategory navigation displays matching products</x:v>
+      </x:c>
+      <x:c r="F33" s="98" t="str">
+        <x:v>Automation Exercise home page is available.</x:v>
+      </x:c>
+      <x:c r="G33" s="98" t="str">
+        <x:v>Women &gt; Dress and Men &gt; Tshirts category examples.</x:v>
+      </x:c>
+      <x:c r="H33" s="98" t="str">
+        <x:v>1. Verify the Category panel is visible.
+2. Expand Women and select Dress.
+3. Verify the Women - Dress Products heading and relevant products.
+4. Expand Men and select Tshirts.
+5. Verify the Men - Tshirts Products heading and relevant products.</x:v>
+      </x:c>
+      <x:c r="I33" s="98" t="str">
+        <x:v>Each selected subcategory opens the correct category page and displays products belonging to that selection.</x:v>
+      </x:c>
+      <x:c r="J33" s="98" t="str"/>
+      <x:c r="K33" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L33" s="102" t="str"/>
+      <x:c r="M33" s="103" t="str"/>
+      <x:c r="N33" s="102" t="str"/>
+      <x:c r="O33" s="102" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P33" s="98" t="str">
+        <x:v>Jira AEQA-110; linked to AEQA-18. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q33" s="100" t="str">
+        <x:v>REQ-CATALOG-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="112.5" customHeight="1">
+      <x:c r="A34" s="112" t="str">
+        <x:v>AE-CATALOG-002</x:v>
+      </x:c>
+      <x:c r="B34" s="95" t="str">
+        <x:v>Products</x:v>
+      </x:c>
+      <x:c r="C34" s="95" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D34" s="95" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E34" s="91" t="str">
+        <x:v>Verify brand navigation and switching displays products for the selected brand</x:v>
+      </x:c>
+      <x:c r="F34" s="91" t="str">
+        <x:v>Automation Exercise Products page is available.</x:v>
+      </x:c>
+      <x:c r="G34" s="91" t="str">
+        <x:v>Two brands shown in the Brands panel, such as Polo and H&amp;M.</x:v>
+      </x:c>
+      <x:c r="H34" s="91" t="str">
+        <x:v>1. Open Products and verify the Brands panel.
+2. Select the first brand and verify the brand-products heading and results.
+3. Select a different brand.
+4. Verify the heading and results update to the second brand.</x:v>
+      </x:c>
+      <x:c r="I34" s="91" t="str">
+        <x:v>The selected brand name is shown and only its brand-product results are displayed after each switch.</x:v>
+      </x:c>
+      <x:c r="J34" s="91" t="str"/>
+      <x:c r="K34" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L34" s="95" t="str"/>
+      <x:c r="M34" s="96" t="str"/>
+      <x:c r="N34" s="95" t="str"/>
+      <x:c r="O34" s="95" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P34" s="91" t="str">
+        <x:v>Jira AEQA-111; linked to AEQA-19. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q34" s="93" t="str">
+        <x:v>REQ-CATALOG-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="112.5" customHeight="1">
+      <x:c r="A35" s="113" t="str">
+        <x:v>AE-CART-004</x:v>
+      </x:c>
+      <x:c r="B35" s="102" t="str">
+        <x:v>Cart</x:v>
+      </x:c>
+      <x:c r="C35" s="102" t="str">
+        <x:v>Regression</x:v>
+      </x:c>
+      <x:c r="D35" s="102" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="E35" s="98" t="str">
+        <x:v>Verify searched products remain in the cart after login</x:v>
+      </x:c>
+      <x:c r="F35" s="98" t="str">
+        <x:v>A dedicated QA account exists and is logged out; cart is empty.</x:v>
+      </x:c>
+      <x:c r="G35" s="98" t="str">
+        <x:v>Search term matching multiple products; valid QA credentials.</x:v>
+      </x:c>
+      <x:c r="H35" s="98" t="str">
+        <x:v>1. Open Products and search for a product term.
+2. Verify Searched Products and add visible results to the cart.
+3. Open Cart and record the products.
+4. Select Signup / Login and authenticate.
+5. Return to Cart.
+6. Compare product names, prices, quantities, and totals with the pre-login cart.</x:v>
+      </x:c>
+      <x:c r="I35" s="98" t="str">
+        <x:v>All products added before login remain in the cart with unchanged details after authentication.</x:v>
+      </x:c>
+      <x:c r="J35" s="98" t="str"/>
+      <x:c r="K35" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L35" s="102" t="str"/>
+      <x:c r="M35" s="103" t="str"/>
+      <x:c r="N35" s="102" t="str"/>
+      <x:c r="O35" s="102" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P35" s="98" t="str">
+        <x:v>Jira AEQA-112; linked to AEQA-20. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q35" s="100" t="str">
+        <x:v>REQ-CART-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="112.5" customHeight="1">
+      <x:c r="A36" s="112" t="str">
+        <x:v>AE-REVIEW-001</x:v>
+      </x:c>
+      <x:c r="B36" s="95" t="str">
+        <x:v>Products</x:v>
+      </x:c>
+      <x:c r="C36" s="95" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D36" s="95" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E36" s="91" t="str">
+        <x:v>Verify a visitor can submit a review from a product-details page</x:v>
+      </x:c>
+      <x:c r="F36" s="91" t="str">
+        <x:v>Automation Exercise Products page is available.</x:v>
+      </x:c>
+      <x:c r="G36" s="91" t="str">
+        <x:v>QA reviewer name; disposable QA email; non-sensitive review text.</x:v>
+      </x:c>
+      <x:c r="H36" s="91" t="str">
+        <x:v>1. Open Products and view a product detail.
+2. Scroll to Write Your Review.
+3. Enter name, email, and review text.
+4. Submit the review.
+5. Observe the confirmation message.</x:v>
+      </x:c>
+      <x:c r="I36" s="91" t="str">
+        <x:v>The review is accepted and the Thank you for your review confirmation is displayed.</x:v>
+      </x:c>
+      <x:c r="J36" s="91" t="str"/>
+      <x:c r="K36" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L36" s="95" t="str"/>
+      <x:c r="M36" s="96" t="str"/>
+      <x:c r="N36" s="95" t="str"/>
+      <x:c r="O36" s="95" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P36" s="91" t="str">
+        <x:v>Jira AEQA-113; linked to AEQA-21. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q36" s="93" t="str">
+        <x:v>REQ-REVIEW-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="112.5" customHeight="1">
+      <x:c r="A37" s="113" t="str">
+        <x:v>AE-CART-005</x:v>
+      </x:c>
+      <x:c r="B37" s="102" t="str">
+        <x:v>Cart</x:v>
+      </x:c>
+      <x:c r="C37" s="102" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D37" s="102" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E37" s="98" t="str">
+        <x:v>Verify a product can be added to the cart from Recommended Items</x:v>
+      </x:c>
+      <x:c r="F37" s="98" t="str">
+        <x:v>Automation Exercise home page is available; cart is empty.</x:v>
+      </x:c>
+      <x:c r="G37" s="98" t="str">
+        <x:v>Any product displayed in Recommended Items.</x:v>
+      </x:c>
+      <x:c r="H37" s="98" t="str">
+        <x:v>1. Scroll to Recommended Items.
+2. Verify recommended products are displayed.
+3. Select Add to cart for one recommended product.
+4. Open Cart.
+5. Verify the chosen product and its price, quantity, and total.</x:v>
+      </x:c>
+      <x:c r="I37" s="98" t="str">
+        <x:v>The selected recommended product is present in the cart with correct line details.</x:v>
+      </x:c>
+      <x:c r="J37" s="98" t="str"/>
+      <x:c r="K37" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L37" s="102" t="str"/>
+      <x:c r="M37" s="103" t="str"/>
+      <x:c r="N37" s="102" t="str"/>
+      <x:c r="O37" s="102" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P37" s="98" t="str">
+        <x:v>Jira AEQA-114; linked to AEQA-22. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q37" s="100" t="str">
+        <x:v>REQ-CART-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="112.5" customHeight="1">
+      <x:c r="A38" s="112" t="str">
+        <x:v>AE-ORDER-004</x:v>
+      </x:c>
+      <x:c r="B38" s="95" t="str">
+        <x:v>Checkout</x:v>
+      </x:c>
+      <x:c r="C38" s="95" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D38" s="95" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="E38" s="91" t="str">
+        <x:v>Verify checkout delivery and billing addresses match the registered account</x:v>
+      </x:c>
+      <x:c r="F38" s="91" t="str">
+        <x:v>A registered QA user is logged in and has at least one product in the cart.</x:v>
+      </x:c>
+      <x:c r="G38" s="91" t="str">
+        <x:v>Known QA registration address and one in-stock product.</x:v>
+      </x:c>
+      <x:c r="H38" s="91" t="str">
+        <x:v>1. Proceed from Cart to Checkout.
+2. Compare Delivery Address with the registered account data.
+3. Compare Billing Address with the registered account data.
+4. Verify name, company if supplied, street, city/state/ZIP, country, and phone fields.</x:v>
+      </x:c>
+      <x:c r="I38" s="91" t="str">
+        <x:v>Delivery and billing sections display the correct registered account address details without omissions or unexpected changes.</x:v>
+      </x:c>
+      <x:c r="J38" s="91" t="str"/>
+      <x:c r="K38" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L38" s="95" t="str"/>
+      <x:c r="M38" s="96" t="str"/>
+      <x:c r="N38" s="95" t="str"/>
+      <x:c r="O38" s="95" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P38" s="91" t="str">
+        <x:v>Jira AEQA-115; linked to AEQA-23. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q38" s="93" t="str">
+        <x:v>REQ-ORDER-004</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="112.5" customHeight="1">
+      <x:c r="A39" s="113" t="str">
+        <x:v>AE-ORDER-005</x:v>
+      </x:c>
+      <x:c r="B39" s="102" t="str">
+        <x:v>Checkout</x:v>
+      </x:c>
+      <x:c r="C39" s="102" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D39" s="102" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E39" s="98" t="str">
+        <x:v>Verify an invoice can be downloaded after a successful purchase</x:v>
+      </x:c>
+      <x:c r="F39" s="98" t="str">
+        <x:v>A registered QA user is logged in and can complete checkout.</x:v>
+      </x:c>
+      <x:c r="G39" s="98" t="str">
+        <x:v>One in-stock product and safe test payment data.</x:v>
+      </x:c>
+      <x:c r="H39" s="98" t="str">
+        <x:v>1. Add a product and complete checkout.
+2. Verify the order success message.
+3. Select Download Invoice.
+4. Confirm a file downloads.
+5. Open the invoice and compare order/product details with the completed purchase.
+6. Select Continue.</x:v>
+      </x:c>
+      <x:c r="I39" s="98" t="str">
+        <x:v>A readable invoice downloads after purchase and contains details consistent with the completed order.</x:v>
+      </x:c>
+      <x:c r="J39" s="98" t="str"/>
+      <x:c r="K39" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L39" s="102" t="str"/>
+      <x:c r="M39" s="103" t="str"/>
+      <x:c r="N39" s="102" t="str"/>
+      <x:c r="O39" s="102" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P39" s="98" t="str">
+        <x:v>Jira AEQA-116; linked to AEQA-24. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q39" s="100" t="str">
+        <x:v>REQ-ORDER-005</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="112.5" customHeight="1">
+      <x:c r="A40" s="112" t="str">
+        <x:v>AE-NAV-002</x:v>
+      </x:c>
+      <x:c r="B40" s="95" t="str">
+        <x:v>Navigation</x:v>
+      </x:c>
+      <x:c r="C40" s="95" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D40" s="95" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E40" s="91" t="str">
+        <x:v>Verify scrolling down and returning to the top with the arrow button</x:v>
+      </x:c>
+      <x:c r="F40" s="91" t="str">
+        <x:v>Automation Exercise home page is loaded with enough content to scroll.</x:v>
+      </x:c>
+      <x:c r="G40" s="91" t="str">
+        <x:v>None.</x:v>
+      </x:c>
+      <x:c r="H40" s="91" t="str">
+        <x:v>1. Scroll to the bottom of the home page.
+2. Verify Subscription is visible.
+3. Select the bottom-right scroll-up arrow.
+4. Verify the page returns to the top and the Full-Fledged practice website heading is visible.</x:v>
+      </x:c>
+      <x:c r="I40" s="91" t="str">
+        <x:v>The user can reach the footer and the arrow control returns the page to the top content.</x:v>
+      </x:c>
+      <x:c r="J40" s="91" t="str"/>
+      <x:c r="K40" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L40" s="95" t="str"/>
+      <x:c r="M40" s="96" t="str"/>
+      <x:c r="N40" s="95" t="str"/>
+      <x:c r="O40" s="95" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P40" s="91" t="str">
+        <x:v>Jira AEQA-117; linked to AEQA-25. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q40" s="93" t="str">
+        <x:v>REQ-NAV-002</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="112.5" customHeight="1">
+      <x:c r="A41" s="114" t="str">
+        <x:v>AE-NAV-003</x:v>
+      </x:c>
+      <x:c r="B41" s="109" t="str">
+        <x:v>Navigation</x:v>
+      </x:c>
+      <x:c r="C41" s="109" t="str">
+        <x:v>Functional — Positive</x:v>
+      </x:c>
+      <x:c r="D41" s="109" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E41" s="105" t="str">
+        <x:v>Verify manual scrolling down and back to the top without the arrow button</x:v>
+      </x:c>
+      <x:c r="F41" s="105" t="str">
+        <x:v>Automation Exercise home page is loaded with enough content to scroll.</x:v>
+      </x:c>
+      <x:c r="G41" s="105" t="str">
+        <x:v>None.</x:v>
+      </x:c>
+      <x:c r="H41" s="105" t="str">
+        <x:v>1. Manually scroll to the bottom of the home page without using the arrow control.
+2. Verify Subscription is visible.
+3. Manually scroll back to the top.
+4. Verify the Full-Fledged practice website heading is visible.</x:v>
+      </x:c>
+      <x:c r="I41" s="105" t="str">
+        <x:v>Manual scrolling reaches the footer and returns to the top without using the arrow button.</x:v>
+      </x:c>
+      <x:c r="J41" s="105" t="str"/>
+      <x:c r="K41" s="120" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L41" s="109" t="str"/>
+      <x:c r="M41" s="110" t="str"/>
+      <x:c r="N41" s="109" t="str"/>
+      <x:c r="O41" s="109" t="str">
+        <x:v>NA</x:v>
+      </x:c>
+      <x:c r="P41" s="105" t="str">
+        <x:v>Jira AEQA-118; linked to AEQA-26. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+      </x:c>
+      <x:c r="Q41" s="107" t="str">
+        <x:v>REQ-NAV-003</x:v>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="30"/>
@@ -3702,14 +4410,26 @@
     <x:cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="Not Run"/>
     <x:cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="Retest"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="C8:C17">
       <x:formula1>"Functional — Positive,Functional — Negative,Regression,Smoke,Exploratory, Security — Negative, Security — Authentication, Security — Input Validation"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="B29:B41">
+      <x:formula1>Lists!$D$2:$D$11</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C29:C41">
+      <x:formula1>Lists!$C$2:$C$6</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D29:D41">
+      <x:formula1>Lists!$B$2:$B$5</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K29:K41">
+      <x:formula1>Lists!$A$2:$A$6</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ddc3311e7014e60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb18d153a93f842ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3727,7 +4447,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="48" t="s">
-        <x:v>228</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="B1" s="48"/>
       <x:c r="C1" s="48"/>
@@ -3739,7 +4459,7 @@
     </x:row>
     <x:row r="3" ht="15.5">
       <x:c r="A3" s="49" t="s">
-        <x:v>229</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="B3" s="49"/>
       <x:c r="C3" s="49"/>
@@ -3751,7 +4471,7 @@
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="50" t="s">
-        <x:v>230</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="B4" s="51"/>
       <x:c r="C4" s="51"/>
@@ -3803,184 +4523,184 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="12" t="s">
-        <x:v>231</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="B10" s="12" t="s">
-        <x:v>232</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="C10" s="12" t="s">
-        <x:v>233</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="D10" s="12" t="s">
-        <x:v>234</x:v>
+        <x:v>229</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="34" customHeight="1">
       <x:c r="A11" s="13" t="s">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B11" s="6" t="s">
-        <x:v>235</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C11" s="6" t="s">
-        <x:v>236</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="D11" s="6" t="s">
-        <x:v>237</x:v>
+        <x:v>232</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="34" customHeight="1">
       <x:c r="A12" s="13" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="B12" s="6" t="s">
-        <x:v>235</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C12" s="6" t="s">
-        <x:v>238</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="D12" s="6" t="s">
-        <x:v>239</x:v>
+        <x:v>234</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
       <x:c r="A13" s="13" t="s">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B13" s="6" t="s">
+        <x:v>230</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="s">
         <x:v>235</x:v>
       </x:c>
-      <x:c r="C13" s="6" t="s">
-        <x:v>240</x:v>
-      </x:c>
       <x:c r="D13" s="6" t="s">
-        <x:v>241</x:v>
+        <x:v>236</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
       <x:c r="A14" s="13" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="B14" s="6" t="s">
-        <x:v>235</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C14" s="6" t="s">
-        <x:v>242</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="D14" s="6" t="s">
-        <x:v>243</x:v>
+        <x:v>238</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="34" customHeight="1">
       <x:c r="A15" s="13" t="s">
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B15" s="6" t="s">
-        <x:v>235</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C15" s="6" t="s">
-        <x:v>244</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D15" s="6" t="s">
-        <x:v>245</x:v>
+        <x:v>240</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
       <x:c r="A16" s="13" t="s">
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B16" s="6" t="s">
-        <x:v>246</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="C16" s="6" t="s">
-        <x:v>247</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="D16" s="6" t="s">
-        <x:v>248</x:v>
+        <x:v>243</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="34" customHeight="1">
       <x:c r="A17" s="13" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B17" s="6" t="s">
-        <x:v>235</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C17" s="6" t="s">
-        <x:v>249</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="D17" s="6" t="s">
-        <x:v>250</x:v>
+        <x:v>245</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="34" customHeight="1">
       <x:c r="A18" s="13" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B18" s="6" t="s">
-        <x:v>235</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C18" s="6" t="s">
-        <x:v>251</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="D18" s="6" t="s">
-        <x:v>252</x:v>
+        <x:v>247</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="34" customHeight="1">
       <x:c r="A19" s="13" t="s">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B19" s="6" t="s">
-        <x:v>253</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C19" s="6" t="s">
-        <x:v>254</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="D19" s="6" t="s">
-        <x:v>255</x:v>
+        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="34" customHeight="1">
       <x:c r="A20" s="13" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B20" s="6" t="s">
-        <x:v>253</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="C20" s="6" t="s">
-        <x:v>256</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="D20" s="6" t="s">
-        <x:v>257</x:v>
+        <x:v>252</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="34" customHeight="1">
       <x:c r="A21" s="13" t="s">
-        <x:v>258</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="B21" s="6" t="s">
-        <x:v>259</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="C21" s="6" t="s">
-        <x:v>260</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="D21" s="6" t="s">
-        <x:v>261</x:v>
+        <x:v>256</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="38" customHeight="1">
       <x:c r="A22" s="25" t="s">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B22" s="21" t="s">
-        <x:v>235</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="C22" s="21" t="s">
-        <x:v>262</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="D22" s="21" t="s">
-        <x:v>263</x:v>
+        <x:v>258</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4006,102 +4726,102 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="19" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B1" s="20" t="s">
-        <x:v>10</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C1" s="20" t="s">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D1" s="20" t="s">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E1" s="20" t="s">
-        <x:v>264</x:v>
+        <x:v>259</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="16" t="s">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B2" s="17" t="s">
-        <x:v>41</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C2" s="17" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D2" s="17" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E2" s="18" t="s">
-        <x:v>265</x:v>
+        <x:v>260</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="16" t="s">
-        <x:v>34</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B3" s="17" t="s">
-        <x:v>27</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C3" s="17" t="s">
-        <x:v>51</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D3" s="17" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="E3" s="18" t="s">
-        <x:v>266</x:v>
+        <x:v>261</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="16" t="s">
-        <x:v>107</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B4" s="17" t="s">
-        <x:v>192</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="C4" s="17" t="s">
-        <x:v>267</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="D4" s="17" t="s">
-        <x:v>100</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E4" s="18" t="s">
-        <x:v>268</x:v>
+        <x:v>263</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="16" t="s">
-        <x:v>269</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="B5" s="17" t="s">
-        <x:v>203</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C5" s="17" t="s">
-        <x:v>270</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="D5" s="17" t="s">
-        <x:v>113</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="E5" s="18" t="s">
-        <x:v>271</x:v>
+        <x:v>266</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="16" t="s">
-        <x:v>272</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="B6" s="17"/>
       <x:c r="C6" s="17" t="s">
-        <x:v>273</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="D6" s="21" t="s">
-        <x:v>148</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="E6" s="18" t="s">
-        <x:v>274</x:v>
+        <x:v>269</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
@@ -4109,23 +4829,28 @@
       <x:c r="B7" s="26"/>
       <x:c r="C7" s="26"/>
       <x:c r="D7" s="27" t="s">
-        <x:v>167</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="E7" s="26"/>
     </x:row>
     <x:row r="8">
       <x:c r="D8" t="s">
-        <x:v>191</x:v>
+        <x:v>186</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="D9" t="s">
-        <x:v>202</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="D10" t="s">
-        <x:v>213</x:v>
+        <x:v>208</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="D11" t="str">
+        <x:v>Checkout</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Jira / RTM reconciliation
</commit_message>
<xml_diff>
--- a/Automation Exercise Project/Test Cases/Automation Exercise - Test Case Repository.xlsx
+++ b/Automation Exercise Project/Test Cases/Automation Exercise - Test Case Repository.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="Rb752f6ac4e644024"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="R48bc4ed0262a4b57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R3f1151270f7f4af2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="Rfb6f3c09459a41b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="Reca5500ce29e4ac4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R0f944743fc764298"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1010,10 +1010,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="16">
+  <x:fonts count="17">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -1106,8 +1107,14 @@
       <x:color rgb="FF92400E"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF166534"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="14">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -1172,6 +1179,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFEF3C7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCFCE7"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -1492,7 +1504,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="121">
+  <x:cellXfs count="124">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1846,6 +1858,15 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="15" fillId="13" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="12" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="14" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="14" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2003,9 +2024,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2205,7 +2226,7 @@
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="38" t="n">
         <x:f>COUNTIF(K8:K107,"Pass")</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E5" s="39"/>
       <x:c r="F5" s="2"/>
@@ -2217,7 +2238,7 @@
       <x:c r="I5" s="2"/>
       <x:c r="J5" s="38" t="n">
         <x:f>COUNTIF(K8:K107,"Not Run")</x:f>
-        <x:v>13</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="K5" s="39"/>
       <x:c r="M5" s="43"/>
@@ -3485,18 +3506,26 @@
       <x:c r="I30" s="91" t="str">
         <x:v>The newly registered user completes checkout and sees the order success confirmation.</x:v>
       </x:c>
-      <x:c r="J30" s="91" t="str"/>
-      <x:c r="K30" s="119" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="L30" s="95" t="str"/>
-      <x:c r="M30" s="96" t="str"/>
-      <x:c r="N30" s="95" t="str"/>
+      <x:c r="J30" s="91" t="str">
+        <x:v>The newly registered user completes checkout and sees the order success confirmation.</x:v>
+      </x:c>
+      <x:c r="K30" s="123" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L30" s="95" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="M30" s="121" t="n">
+        <x:v>46245</x:v>
+      </x:c>
+      <x:c r="N30" s="95" t="str">
+        <x:v>..\Screenshots\AE-ORDER-001.png</x:v>
+      </x:c>
       <x:c r="O30" s="95" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="P30" s="91" t="str">
-        <x:v>Jira AEQA-107; linked to AEQA-14. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+        <x:v>Executed in Jira AEQA-107 and passed. Registration during checkout, order placement, and confirmation were verified; screenshot evidence is synchronized locally.</x:v>
       </x:c>
       <x:c r="Q30" s="93" t="str">
         <x:v>REQ-ORDER-001</x:v>
@@ -4429,7 +4458,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb18d153a93f842ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b29d7b0d9a64e1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
rtm jira artifact sync
</commit_message>
<xml_diff>
--- a/Automation Exercise Project/Test Cases/Automation Exercise - Test Case Repository.xlsx
+++ b/Automation Exercise Project/Test Cases/Automation Exercise - Test Case Repository.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="Rfb6f3c09459a41b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="Reca5500ce29e4ac4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R0f944743fc764298"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="R6461755746f44554"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="Rf2ae819dbe4a489b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R87bbe443ef094702"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1504,7 +1504,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="124">
+  <x:cellXfs count="125">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1867,6 +1867,9 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="16" fillId="14" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="11" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2226,7 +2229,7 @@
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="38" t="n">
         <x:f>COUNTIF(K8:K107,"Pass")</x:f>
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E5" s="39"/>
       <x:c r="F5" s="2"/>
@@ -2238,7 +2241,7 @@
       <x:c r="I5" s="2"/>
       <x:c r="J5" s="38" t="n">
         <x:f>COUNTIF(K8:K107,"Not Run")</x:f>
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="K5" s="39"/>
       <x:c r="M5" s="43"/>
@@ -3464,7 +3467,7 @@
         <x:v>NA</x:v>
       </x:c>
       <x:c r="P29" s="84" t="str">
-        <x:v>Jira AEQA-106; linked to AEQA-1. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+        <x:v>Jira AEQA-106 is workflow Done but execution remains Not Run. AEQA-121 tracks Playwright implementation. Do not mark Pass until evidence is produced.</x:v>
       </x:c>
       <x:c r="Q29" s="86" t="str">
         <x:v>REQ-AUTH-001</x:v>
@@ -3665,18 +3668,26 @@
       <x:c r="I33" s="98" t="str">
         <x:v>Each selected subcategory opens the correct category page and displays products belonging to that selection.</x:v>
       </x:c>
-      <x:c r="J33" s="98" t="str"/>
+      <x:c r="J33" s="98" t="str">
+        <x:v>Each selected subcategory opened the correct category page and displayed products belonging to that selection.</x:v>
+      </x:c>
       <x:c r="K33" s="119" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="L33" s="102" t="str"/>
-      <x:c r="M33" s="103" t="str"/>
-      <x:c r="N33" s="102" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L33" s="102" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="M33" s="124" t="n">
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="N33" s="102" t="str">
+        <x:v>Jira native attachment (AEQA-110)</x:v>
+      </x:c>
       <x:c r="O33" s="102" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="P33" s="98" t="str">
-        <x:v>Jira AEQA-110; linked to AEQA-18. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+        <x:v>Executed manually in Jira AEQA-110. Women &gt; Dress and Men &gt; Tshirts headings and matching products were verified.</x:v>
       </x:c>
       <x:c r="Q33" s="100" t="str">
         <x:v>REQ-CATALOG-001</x:v>
@@ -3718,7 +3729,7 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="L34" s="95" t="str"/>
-      <x:c r="M34" s="96" t="str"/>
+      <x:c r="M34" s="121" t="str"/>
       <x:c r="N34" s="95" t="str"/>
       <x:c r="O34" s="95" t="str">
         <x:v>NA</x:v>
@@ -3768,7 +3779,7 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="L35" s="102" t="str"/>
-      <x:c r="M35" s="103" t="str"/>
+      <x:c r="M35" s="124" t="str"/>
       <x:c r="N35" s="102" t="str"/>
       <x:c r="O35" s="102" t="str">
         <x:v>NA</x:v>
@@ -3817,7 +3828,7 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="L36" s="95" t="str"/>
-      <x:c r="M36" s="96" t="str"/>
+      <x:c r="M36" s="121" t="str"/>
       <x:c r="N36" s="95" t="str"/>
       <x:c r="O36" s="95" t="str">
         <x:v>NA</x:v>
@@ -3866,7 +3877,7 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="L37" s="102" t="str"/>
-      <x:c r="M37" s="103" t="str"/>
+      <x:c r="M37" s="124" t="str"/>
       <x:c r="N37" s="102" t="str"/>
       <x:c r="O37" s="102" t="str">
         <x:v>NA</x:v>
@@ -3909,18 +3920,28 @@
       <x:c r="I38" s="91" t="str">
         <x:v>Delivery and billing sections display the correct registered account address details without omissions or unexpected changes.</x:v>
       </x:c>
-      <x:c r="J38" s="91" t="str"/>
+      <x:c r="J38" s="91" t="str">
+        <x:v>Delivery and billing sections displayed the expected registered QA-account name and address details without omissions or unexpected changes.</x:v>
+      </x:c>
       <x:c r="K38" s="119" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="L38" s="95" t="str"/>
-      <x:c r="M38" s="96" t="str"/>
-      <x:c r="N38" s="95" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L38" s="95" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="M38" s="121" t="n">
+        <x:v>46249</x:v>
+      </x:c>
+      <x:c r="N38" s="95" t="str">
+        <x:v>..\Automation\Execution Evidence\AE-ORDER-004.png
+..\Automation\Execution Evidence\AE-ORDER-004-evidence.html
+..\Automation\Execution Evidence\AE-ORDER-004-evidence.pdf</x:v>
+      </x:c>
       <x:c r="O38" s="95" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="P38" s="91" t="str">
-        <x:v>Jira AEQA-115; linked to AEQA-23. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+        <x:v>Passed manually in Jira AEQA-115 and automated under AEQA-102 / AEQA-105. Evidence synchronized on 2026-08-16.</x:v>
       </x:c>
       <x:c r="Q38" s="93" t="str">
         <x:v>REQ-ORDER-004</x:v>
@@ -4458,7 +4479,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b29d7b0d9a64e1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb90ddaaaa80a4351"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs: reconcile Jira and portfolio artifacts
Reconcile completed registration, checkout, cart persistence, and product review results across Jira, the RTM, the Test Case Repository, evidence, and README documentation.

Complete the planned automation Test Case fields for AEQA-125 through AEQA-128 while keeping them Backlog and Not Run.
</commit_message>
<xml_diff>
--- a/Automation Exercise Project/Test Cases/Automation Exercise - Test Case Repository.xlsx
+++ b/Automation Exercise Project/Test Cases/Automation Exercise - Test Case Repository.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="R04130030fae94006"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="R4cc49c53546a4988"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rdb44b5af0fee44f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="1" r:id="Rd2c02e89885c41d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" r:id="R890344f8f5694c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R95b0b5f3008a451f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2227,19 +2227,17 @@
       <x:c r="B5" s="39"/>
       <x:c r="C5" s="2"/>
       <x:c r="D5" s="38" t="n">
-        <x:f>COUNTIF(K8:K107,"Pass")</x:f>
-        <x:v>22</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E5" s="39"/>
       <x:c r="F5" s="2"/>
       <x:c r="G5" s="38" t="n">
-        <x:f>COUNTIF(K8:K107,"Fail")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="H5" s="39"/>
       <x:c r="I5" s="2"/>
       <x:c r="J5" s="38" t="n">
-        <x:v>15</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="K5" s="39"/>
       <x:c r="M5" s="43"/>
@@ -3454,18 +3452,26 @@
       <x:c r="I29" s="84" t="str">
         <x:v>The account is created successfully, the user is authenticated, optional selections do not block registration, and cleanup succeeds.</x:v>
       </x:c>
-      <x:c r="J29" s="84" t="str"/>
+      <x:c r="J29" s="84" t="str">
+        <x:v>Pass. The complete registration workflow succeeded, including both optional subscription selections, authenticated state, and account cleanup.</x:v>
+      </x:c>
       <x:c r="K29" s="118" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="L29" s="88" t="str"/>
-      <x:c r="M29" s="89" t="str"/>
-      <x:c r="N29" s="88" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L29" s="88" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="M29" s="89" t="str">
+        <x:v>2026-08-17</x:v>
+      </x:c>
+      <x:c r="N29" s="88" t="str">
+        <x:v>..\Automation\Execution Evidence\AE-SIGNUP-006.png; Jira AEQA-106 attachment: AE-SIGNUP-006-automation.png</x:v>
+      </x:c>
       <x:c r="O29" s="88" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="P29" s="84" t="str">
-        <x:v>Jira AEQA-106 is workflow Done but execution remains Not Run. AEQA-121 tracks Playwright implementation. Do not mark Pass until evidence is produced.</x:v>
+        <x:v>Jira AEQA-106 passed and is linked to AEQA-1 / REQ-AUTH-001. Playwright implementation AEQA-121 is Done, and evidence is attached.</x:v>
       </x:c>
       <x:c r="Q29" s="86" t="str">
         <x:v>REQ-AUTH-001</x:v>
@@ -3567,18 +3573,26 @@
       <x:c r="I31" s="98" t="str">
         <x:v>A user registered before shopping can place the order successfully and receives confirmation.</x:v>
       </x:c>
-      <x:c r="J31" s="98" t="str"/>
+      <x:c r="J31" s="98" t="str">
+        <x:v>Pass. A user registered before shopping, completed checkout, and received the order confirmation.</x:v>
+      </x:c>
       <x:c r="K31" s="119" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="L31" s="102" t="str"/>
-      <x:c r="M31" s="103" t="str"/>
-      <x:c r="N31" s="102" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L31" s="102" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="M31" s="103" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="N31" s="102" t="str">
+        <x:v>Jira AEQA-108 attachments: three screenshots and invoice (1).txt</x:v>
+      </x:c>
       <x:c r="O31" s="102" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="P31" s="98" t="str">
-        <x:v>Jira AEQA-108; linked to AEQA-15. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+        <x:v>Jira AEQA-108 passed and is linked to AEQA-15 / REQ-ORDER-002. Evidence and invoice output are attached to the Jira Test Case.</x:v>
       </x:c>
       <x:c r="Q31" s="100" t="str">
         <x:v>REQ-ORDER-002</x:v>
@@ -3617,18 +3631,26 @@
       <x:c r="I32" s="91" t="str">
         <x:v>The authenticated user completes checkout and sees the order success confirmation.</x:v>
       </x:c>
-      <x:c r="J32" s="91" t="str"/>
+      <x:c r="J32" s="91" t="str">
+        <x:v>Pass. The authenticated user completed checkout and received the order success confirmation.</x:v>
+      </x:c>
       <x:c r="K32" s="119" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="L32" s="95" t="str"/>
-      <x:c r="M32" s="96" t="str"/>
-      <x:c r="N32" s="95" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L32" s="95" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="M32" s="96" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="N32" s="95" t="str">
+        <x:v>Jira AEQA-109 attachments: three screenshots and invoice (2).txt</x:v>
+      </x:c>
       <x:c r="O32" s="95" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="P32" s="91" t="str">
-        <x:v>Jira AEQA-109; linked to AEQA-16. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+        <x:v>Jira AEQA-109 passed and is linked to AEQA-16 / REQ-ORDER-003. Evidence and invoice output are attached to the Jira Test Case.</x:v>
       </x:c>
       <x:c r="Q32" s="93" t="str">
         <x:v>REQ-ORDER-003</x:v>
@@ -3772,18 +3794,26 @@
       <x:c r="I35" s="98" t="str">
         <x:v>All products added before login remain in the cart with unchanged details after authentication.</x:v>
       </x:c>
-      <x:c r="J35" s="98" t="str"/>
+      <x:c r="J35" s="98" t="str">
+        <x:v>Pass. The searched products remained in the cart after login with the expected names, prices, quantities, and totals.</x:v>
+      </x:c>
       <x:c r="K35" s="119" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="L35" s="102" t="str"/>
-      <x:c r="M35" s="124" t="str"/>
-      <x:c r="N35" s="102" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L35" s="102" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="M35" s="124" t="str">
+        <x:v>2026-08-17</x:v>
+      </x:c>
+      <x:c r="N35" s="102" t="str">
+        <x:v>Jira AEQA-112 attachments: AE-CART-004(1).png and AE-CART-004(2).png</x:v>
+      </x:c>
       <x:c r="O35" s="102" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="P35" s="98" t="str">
-        <x:v>Jira AEQA-112; linked to AEQA-20. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+        <x:v>Jira AEQA-112 passed and is linked to AEQA-20 / REQ-CART-004. Manual evidence is attached to AEQA-112, and separate Playwright evidence is attached to AEQA-122.</x:v>
       </x:c>
       <x:c r="Q35" s="100" t="str">
         <x:v>REQ-CART-004</x:v>
@@ -3821,18 +3851,26 @@
       <x:c r="I36" s="91" t="str">
         <x:v>The review is accepted and the Thank you for your review confirmation is displayed.</x:v>
       </x:c>
-      <x:c r="J36" s="91" t="str"/>
+      <x:c r="J36" s="91" t="str">
+        <x:v>Pass. A visitor submitted the review and the Thank you for your review confirmation was displayed.</x:v>
+      </x:c>
       <x:c r="K36" s="119" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="L36" s="95" t="str"/>
-      <x:c r="M36" s="121" t="str"/>
-      <x:c r="N36" s="95" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L36" s="95" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="M36" s="121" t="str">
+        <x:v>2026-08-17</x:v>
+      </x:c>
+      <x:c r="N36" s="95" t="str">
+        <x:v>Jira AEQA-113 attachments (2 manual screenshots)</x:v>
+      </x:c>
       <x:c r="O36" s="95" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="P36" s="91" t="str">
-        <x:v>Jira AEQA-113; linked to AEQA-21. Execute in QA and synchronize result, evidence, and defects back to Jira and the RTM.</x:v>
+        <x:v>Jira AEQA-113 passed and is linked to AEQA-21 / REQ-REVIEW-001. Manual evidence is attached to AEQA-113.</x:v>
       </x:c>
       <x:c r="Q36" s="93" t="str">
         <x:v>REQ-REVIEW-001</x:v>
@@ -4112,7 +4150,7 @@
 2. No authenticated account is required.</x:v>
       </x:c>
       <x:c r="G42" s="30" t="str">
-        <x:v>Generated synthetic name and email address; non-sensitive automated QA review text.</x:v>
+        <x:v>Random synthetic reviewer name and email address; review text: QA By The McMahon Standard.</x:v>
       </x:c>
       <x:c r="H42" s="30" t="str">
         <x:v>1. Open https://automationexercise.com and select Products.
@@ -4126,18 +4164,27 @@
       <x:c r="I42" s="30" t="str">
         <x:v>Product details and the review form load, the populated review is accepted, and the exact success message is displayed.</x:v>
       </x:c>
-      <x:c r="J42" s="30" t="str"/>
+      <x:c r="J42" s="30" t="str">
+        <x:v>Pass. Playwright generated a random name and email, submitted QA By The McMahon Standard, and displayed the exact success confirmation.</x:v>
+      </x:c>
       <x:c r="K42" s="30" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="L42" s="30" t="str"/>
-      <x:c r="M42" s="31" t="str"/>
-      <x:c r="N42" s="30" t="str"/>
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="L42" s="30" t="str">
+        <x:v>KM</x:v>
+      </x:c>
+      <x:c r="M42" s="31" t="str">
+        <x:v>2026-08-17</x:v>
+      </x:c>
+      <x:c r="N42" s="30" t="str">
+        <x:v>..\Automation\Execution Evidence\AE-REVIEW-001(1).png
+..\Automation\Execution Evidence\AE-REVIEW-001(2).png</x:v>
+      </x:c>
       <x:c r="O42" s="30" t="str">
         <x:v>NA</x:v>
       </x:c>
       <x:c r="P42" s="30" t="str">
-        <x:v>Jira AEQA-124; linked to AEQA-21 / REQ-REVIEW-001. Playwright automation planned; attach the HTML report and form/success screenshots after execution.</x:v>
+        <x:v>Jira AEQA-124 passed and is linked to AEQA-21 / REQ-REVIEW-001. Playwright uses the shared page object model. The HTML report and two named screenshots provide the automation evidence.</x:v>
       </x:c>
       <x:c r="Q42" s="30" t="str">
         <x:v>REQ-REVIEW-001</x:v>
@@ -4643,7 +4690,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcaefea0b548a49ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ab11cd450624b15"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>